<commit_message>
make smae changes and fixed some bugs
</commit_message>
<xml_diff>
--- a/output/nbo_master_dataset.xlsx
+++ b/output/nbo_master_dataset.xlsx
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -575,14 +575,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ2"/>
+  <dimension ref="A1:AQ3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
@@ -592,8 +592,8 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="42" customWidth="1" min="15" max="15"/>
-    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="39" customWidth="1" min="15" max="15"/>
+    <col width="36" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="18" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
@@ -611,7 +611,7 @@
     <col width="16" customWidth="1" min="31" max="31"/>
     <col width="13" customWidth="1" min="32" max="32"/>
     <col width="18" customWidth="1" min="33" max="33"/>
-    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
     <col width="16" customWidth="1" min="35" max="35"/>
     <col width="16" customWidth="1" min="36" max="36"/>
     <col width="16" customWidth="1" min="37" max="37"/>
@@ -620,7 +620,7 @@
     <col width="20" customWidth="1" min="40" max="40"/>
     <col width="12" customWidth="1" min="41" max="41"/>
     <col width="19" customWidth="1" min="42" max="42"/>
-    <col width="20" customWidth="1" min="43" max="43"/>
+    <col width="42" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -843,83 +843,268 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>SME Products (conventional) Alfalah Milkat Finance</t>
+          <t>IGI Life – WTO Danish Plan Danish Plan</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>BNK</t>
+          <t>IBG</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Conv SME</t>
+          <t>Banca Takaful</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Financing</t>
+          <t>Savings</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>SME Products (conventional) Alfalah Milkat Finance</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
       <c r="N2" s="3" t="n"/>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>SME Products (conventional) Alfalah Milkat Finance</t>
+          <t>IGI LIFE WTO Danish Education Plan</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>SME Products (conventional) Alfalah Milkat Finance</t>
-        </is>
-      </c>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="3" t="n"/>
-      <c r="U2" s="3" t="n"/>
-      <c r="V2" s="3" t="n"/>
-      <c r="W2" s="3" t="n"/>
-      <c r="X2" s="3" t="n"/>
-      <c r="Y2" s="3" t="n"/>
-      <c r="Z2" s="3" t="n"/>
-      <c r="AA2" s="3" t="n"/>
-      <c r="AB2" s="3" t="n"/>
-      <c r="AC2" s="3" t="n"/>
-      <c r="AD2" s="3" t="n"/>
-      <c r="AE2" s="3" t="n"/>
-      <c r="AF2" s="3" t="n"/>
-      <c r="AG2" s="3" t="n"/>
+          <t>IGI LIFE WTO Danish Education Plan</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>NAN</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="AA2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="AB2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AD2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="AE2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AF2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AG2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
       <c r="AH2" s="3" t="inlineStr">
         <is>
-          <t>2 Y To 15 Y</t>
-        </is>
-      </c>
-      <c r="AI2" s="3" t="n"/>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AI2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
       <c r="AJ2" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="AK2" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="AL2" s="3" t="n"/>
-      <c r="AM2" s="3" t="n"/>
-      <c r="AN2" s="3" t="n"/>
-      <c r="AO2" s="3" t="n"/>
-      <c r="AP2" s="3" t="n"/>
-      <c r="AQ2" s="3" t="n"/>
+        <v>25</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="AM2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AN2" s="3" t="n">
+        <v/>
+      </c>
+      <c r="AO2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AP2" s="3" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AQ2" s="3" t="inlineStr">
+        <is>
+          <t>Free 14-day Look Period To Review Policy Terms; Conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Zaamin Takaful Plan</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+      <c r="K3" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="M3" s="5" t="n"/>
+      <c r="N3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>Alfalah Insurance Zaamin Takaful Plan</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>Debit Card</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="n"/>
+      <c r="R3" s="5" t="n"/>
+      <c r="S3" s="5" t="n"/>
+      <c r="T3" s="5" t="n"/>
+      <c r="U3" s="5" t="n"/>
+      <c r="V3" s="5" t="n"/>
+      <c r="W3" s="5" t="n"/>
+      <c r="X3" s="5" t="n"/>
+      <c r="Y3" s="5" t="n"/>
+      <c r="Z3" s="5" t="n"/>
+      <c r="AA3" s="5" t="n"/>
+      <c r="AB3" s="5" t="n"/>
+      <c r="AC3" s="5" t="n"/>
+      <c r="AD3" s="5" t="n"/>
+      <c r="AE3" s="5" t="n"/>
+      <c r="AF3" s="5" t="n"/>
+      <c r="AG3" s="5" t="n"/>
+      <c r="AH3" s="5" t="n"/>
+      <c r="AI3" s="5" t="n"/>
+      <c r="AJ3" s="5" t="n"/>
+      <c r="AK3" s="5" t="n"/>
+      <c r="AL3" s="5" t="n"/>
+      <c r="AM3" s="5" t="n"/>
+      <c r="AN3" s="5" t="n"/>
+      <c r="AO3" s="5" t="n"/>
+      <c r="AP3" s="5" t="n"/>
+      <c r="AQ3" s="5" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AQ1"/>

</xml_diff>

<commit_message>
add time for ratlimit
</commit_message>
<xml_diff>
--- a/output/nbo_master_dataset.xlsx
+++ b/output/nbo_master_dataset.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Use MASTER_DATASET as the base training table. Blank cells indicate attributes not explicitly identified in the source batch.</t>
+          <t>Use MASTER_DATASET as the base training table. Blank cells indicate attributes that could not be safely extracted or inferred.</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -556,7 +556,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>BNK/IBG are inferred from the product family and source folder. Re-run export to upsert matching products.</t>
+          <t>BNK/IBG are inferred from the product family and source folder. Compact inferred values are used when the document strongly implies a field.</t>
         </is>
       </c>
     </row>
@@ -575,14 +575,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ3"/>
+  <dimension ref="A1:AQ19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
@@ -592,11 +592,11 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
-    <col width="39" customWidth="1" min="15" max="15"/>
-    <col width="36" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
     <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="15" customWidth="1" min="22" max="22"/>
@@ -607,8 +607,8 @@
     <col width="16" customWidth="1" min="27" max="27"/>
     <col width="18" customWidth="1" min="28" max="28"/>
     <col width="19" customWidth="1" min="29" max="29"/>
-    <col width="17" customWidth="1" min="30" max="30"/>
-    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="19" customWidth="1" min="31" max="31"/>
     <col width="13" customWidth="1" min="32" max="32"/>
     <col width="18" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
@@ -892,10 +892,10 @@
         </is>
       </c>
       <c r="K2" s="3" t="n">
-        <v/>
+        <v>18</v>
       </c>
       <c r="L2" s="3" t="n">
-        <v/>
+        <v>25</v>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
@@ -943,32 +943,18 @@
           <t>Nan</t>
         </is>
       </c>
-      <c r="W2" s="3" t="n">
-        <v/>
-      </c>
-      <c r="X2" s="3" t="n">
-        <v/>
-      </c>
-      <c r="Y2" s="3" t="n">
-        <v/>
-      </c>
-      <c r="Z2" s="3" t="n">
-        <v/>
-      </c>
-      <c r="AA2" s="3" t="n">
-        <v/>
-      </c>
-      <c r="AB2" s="3" t="n">
-        <v/>
-      </c>
+      <c r="W2" s="3" t="n"/>
+      <c r="X2" s="3" t="n"/>
+      <c r="Y2" s="3" t="n"/>
+      <c r="Z2" s="3" t="n"/>
+      <c r="AA2" s="3" t="n"/>
+      <c r="AB2" s="3" t="n"/>
       <c r="AC2" s="3" t="inlineStr">
         <is>
           <t>Nan</t>
         </is>
       </c>
-      <c r="AD2" s="3" t="n">
-        <v/>
-      </c>
+      <c r="AD2" s="3" t="n"/>
       <c r="AE2" s="3" t="inlineStr">
         <is>
           <t>Nan</t>
@@ -1000,17 +986,13 @@
       <c r="AK2" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="AL2" s="3" t="n">
-        <v/>
-      </c>
+      <c r="AL2" s="3" t="n"/>
       <c r="AM2" s="3" t="inlineStr">
         <is>
           <t>Nan</t>
         </is>
       </c>
-      <c r="AN2" s="3" t="n">
-        <v/>
-      </c>
+      <c r="AN2" s="3" t="n"/>
       <c r="AO2" s="3" t="inlineStr">
         <is>
           <t>Nan</t>
@@ -1053,58 +1035,1560 @@
           <t>Health</t>
         </is>
       </c>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
       <c r="K3" s="5" t="n">
         <v>18</v>
       </c>
       <c r="L3" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="M3" s="5" t="n"/>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
       <c r="N3" s="5" t="n">
         <v>1</v>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
-          <t>Alfalah Insurance Zaamin Takaful Plan</t>
+          <t>Takaful</t>
         </is>
       </c>
       <c r="P3" s="5" t="inlineStr">
         <is>
-          <t>Debit Card</t>
-        </is>
-      </c>
-      <c r="Q3" s="5" t="n"/>
-      <c r="R3" s="5" t="n"/>
-      <c r="S3" s="5" t="n"/>
-      <c r="T3" s="5" t="n"/>
-      <c r="U3" s="5" t="n"/>
-      <c r="V3" s="5" t="n"/>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>NAN</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
       <c r="W3" s="5" t="n"/>
       <c r="X3" s="5" t="n"/>
       <c r="Y3" s="5" t="n"/>
       <c r="Z3" s="5" t="n"/>
       <c r="AA3" s="5" t="n"/>
       <c r="AB3" s="5" t="n"/>
-      <c r="AC3" s="5" t="n"/>
+      <c r="AC3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
       <c r="AD3" s="5" t="n"/>
-      <c r="AE3" s="5" t="n"/>
-      <c r="AF3" s="5" t="n"/>
-      <c r="AG3" s="5" t="n"/>
-      <c r="AH3" s="5" t="n"/>
-      <c r="AI3" s="5" t="n"/>
+      <c r="AE3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AF3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AG3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AH3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AI3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
       <c r="AJ3" s="5" t="n"/>
       <c r="AK3" s="5" t="n"/>
       <c r="AL3" s="5" t="n"/>
-      <c r="AM3" s="5" t="n"/>
+      <c r="AM3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
       <c r="AN3" s="5" t="n"/>
-      <c r="AO3" s="5" t="n"/>
-      <c r="AP3" s="5" t="n"/>
-      <c r="AQ3" s="5" t="n"/>
+      <c r="AO3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AP3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+      <c r="AQ3" s="5" t="inlineStr">
+        <is>
+          <t>Nan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Islamic Banking Free Takaful Coverage</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Islamic Banking</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Islamic Banking Free Takaful Coverage</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Islamic Banking Free Takaful Coverage</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="n"/>
+      <c r="U4" s="3" t="n"/>
+      <c r="V4" s="3" t="n"/>
+      <c r="W4" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="X4" s="3" t="n"/>
+      <c r="Y4" s="3" t="n"/>
+      <c r="Z4" s="3" t="n"/>
+      <c r="AA4" s="3" t="n"/>
+      <c r="AB4" s="3" t="n"/>
+      <c r="AC4" s="3" t="n"/>
+      <c r="AD4" s="3" t="n">
+        <v>25000</v>
+      </c>
+      <c r="AE4" s="3" t="n"/>
+      <c r="AF4" s="3" t="n"/>
+      <c r="AG4" s="3" t="n"/>
+      <c r="AH4" s="3" t="n"/>
+      <c r="AI4" s="3" t="n"/>
+      <c r="AJ4" s="3" t="n"/>
+      <c r="AK4" s="3" t="n"/>
+      <c r="AL4" s="3" t="n"/>
+      <c r="AM4" s="3" t="n"/>
+      <c r="AN4" s="3" t="n"/>
+      <c r="AO4" s="3" t="n"/>
+      <c r="AP4" s="3" t="n"/>
+      <c r="AQ4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Orbits</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>BNK</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Orbits</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Orbit Tier</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Product Utilization</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="5" t="n"/>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Digital</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>Product Sign-up</t>
+        </is>
+      </c>
+      <c r="T5" s="5" t="inlineStr">
+        <is>
+          <t>Orbit</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>RUPEE</t>
+        </is>
+      </c>
+      <c r="V5" s="5" t="n"/>
+      <c r="W5" s="5" t="n"/>
+      <c r="X5" s="5" t="n"/>
+      <c r="Y5" s="5" t="n"/>
+      <c r="Z5" s="5" t="n"/>
+      <c r="AA5" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB5" s="5" t="n"/>
+      <c r="AC5" s="5" t="n"/>
+      <c r="AD5" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="AE5" s="5" t="n"/>
+      <c r="AF5" s="5" t="n"/>
+      <c r="AG5" s="5" t="n"/>
+      <c r="AH5" s="5" t="n"/>
+      <c r="AI5" s="5" t="n"/>
+      <c r="AJ5" s="5" t="n"/>
+      <c r="AK5" s="5" t="n"/>
+      <c r="AL5" s="5" t="n"/>
+      <c r="AM5" s="5" t="n"/>
+      <c r="AN5" s="5" t="n"/>
+      <c r="AO5" s="5" t="n"/>
+      <c r="AP5" s="5" t="inlineStr">
+        <is>
+          <t>9999</t>
+        </is>
+      </c>
+      <c r="AQ5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Orbit Reward Program</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Orbits</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Reward Program</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Mutual Fund Policies</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr">
+        <is>
+          <t>Internet Banking</t>
+        </is>
+      </c>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>Investment</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>Orbit</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="V6" s="3" t="inlineStr">
+        <is>
+          <t>Fiat</t>
+        </is>
+      </c>
+      <c r="W6" s="3" t="n"/>
+      <c r="X6" s="3" t="n"/>
+      <c r="Y6" s="3" t="n"/>
+      <c r="Z6" s="3" t="n"/>
+      <c r="AA6" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="AB6" s="3" t="n"/>
+      <c r="AC6" s="3" t="n"/>
+      <c r="AD6" s="3" t="n"/>
+      <c r="AE6" s="3" t="n"/>
+      <c r="AF6" s="3" t="n"/>
+      <c r="AG6" s="3" t="n"/>
+      <c r="AH6" s="3" t="n"/>
+      <c r="AI6" s="3" t="n"/>
+      <c r="AJ6" s="3" t="n"/>
+      <c r="AK6" s="3" t="n"/>
+      <c r="AL6" s="3" t="n"/>
+      <c r="AM6" s="3" t="n"/>
+      <c r="AN6" s="3" t="n"/>
+      <c r="AO6" s="3" t="n"/>
+      <c r="AP6" s="3" t="inlineStr">
+        <is>
+          <t>9999</t>
+        </is>
+      </c>
+      <c r="AQ6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Convetional Debit Card</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>BNK</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Conv Consumer</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="5" t="n"/>
+      <c r="O7" s="5" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="inlineStr">
+        <is>
+          <t>Debit</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Mobile App</t>
+        </is>
+      </c>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="5" t="n"/>
+      <c r="T7" s="5" t="n"/>
+      <c r="U7" s="5" t="n"/>
+      <c r="V7" s="5" t="n"/>
+      <c r="W7" s="5" t="n"/>
+      <c r="X7" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="Y7" s="5" t="n"/>
+      <c r="Z7" s="5" t="n"/>
+      <c r="AA7" s="5" t="n"/>
+      <c r="AB7" s="5" t="n"/>
+      <c r="AC7" s="5" t="n"/>
+      <c r="AD7" s="5" t="n"/>
+      <c r="AE7" s="5" t="n"/>
+      <c r="AF7" s="5" t="n"/>
+      <c r="AG7" s="5" t="n"/>
+      <c r="AH7" s="5" t="n"/>
+      <c r="AI7" s="5" t="n"/>
+      <c r="AJ7" s="5" t="n"/>
+      <c r="AK7" s="5" t="n"/>
+      <c r="AL7" s="5" t="n"/>
+      <c r="AM7" s="5" t="n"/>
+      <c r="AN7" s="5" t="n"/>
+      <c r="AO7" s="5" t="n"/>
+      <c r="AP7" s="5" t="n"/>
+      <c r="AQ7" s="5" t="inlineStr">
+        <is>
+          <t>Daily Limits, Min &amp; Max Financing Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Zindagi Premier Takaful Savings Plan</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="L8" s="3" t="n"/>
+      <c r="M8" s="3" t="n"/>
+      <c r="N8" s="3" t="n"/>
+      <c r="O8" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Zindagi Premier Takaful Savings Plan</t>
+        </is>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Zindagi Premier Takaful Savings Plan</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="n"/>
+      <c r="R8" s="3" t="n"/>
+      <c r="S8" s="3" t="n"/>
+      <c r="T8" s="3" t="n"/>
+      <c r="U8" s="3" t="inlineStr">
+        <is>
+          <t>PKR</t>
+        </is>
+      </c>
+      <c r="V8" s="3" t="n"/>
+      <c r="W8" s="3" t="n"/>
+      <c r="X8" s="3" t="n"/>
+      <c r="Y8" s="3" t="n"/>
+      <c r="Z8" s="3" t="n"/>
+      <c r="AA8" s="3" t="n"/>
+      <c r="AB8" s="3" t="n">
+        <v>15000</v>
+      </c>
+      <c r="AC8" s="3" t="n"/>
+      <c r="AD8" s="3" t="n"/>
+      <c r="AE8" s="3" t="inlineStr">
+        <is>
+          <t>Unit Link</t>
+        </is>
+      </c>
+      <c r="AF8" s="3" t="inlineStr">
+        <is>
+          <t>Bonus Based</t>
+        </is>
+      </c>
+      <c r="AG8" s="3" t="n"/>
+      <c r="AH8" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="AI8" s="3" t="n"/>
+      <c r="AJ8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="AK8" s="3" t="n"/>
+      <c r="AL8" s="3" t="n"/>
+      <c r="AM8" s="3" t="n"/>
+      <c r="AN8" s="3" t="n"/>
+      <c r="AO8" s="3" t="n"/>
+      <c r="AP8" s="3" t="n"/>
+      <c r="AQ8" s="3" t="inlineStr">
+        <is>
+          <t>14 Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>WTO Danish Plan</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="M9" s="5" t="n"/>
+      <c r="N9" s="5" t="n"/>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Danish Education Plan</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Danish Education Plan</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="n"/>
+      <c r="R9" s="5" t="n"/>
+      <c r="S9" s="5" t="n"/>
+      <c r="T9" s="5" t="n"/>
+      <c r="U9" s="5" t="n"/>
+      <c r="V9" s="5" t="n"/>
+      <c r="W9" s="5" t="n"/>
+      <c r="X9" s="5" t="n"/>
+      <c r="Y9" s="5" t="n"/>
+      <c r="Z9" s="5" t="n"/>
+      <c r="AA9" s="5" t="n"/>
+      <c r="AB9" s="5" t="n"/>
+      <c r="AC9" s="5" t="n"/>
+      <c r="AD9" s="5" t="n"/>
+      <c r="AE9" s="5" t="n"/>
+      <c r="AF9" s="5" t="n"/>
+      <c r="AG9" s="5" t="n"/>
+      <c r="AH9" s="5" t="inlineStr">
+        <is>
+          <t>10-25 Y</t>
+        </is>
+      </c>
+      <c r="AI9" s="5" t="n"/>
+      <c r="AJ9" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="AK9" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="AL9" s="5" t="n"/>
+      <c r="AM9" s="5" t="n"/>
+      <c r="AN9" s="5" t="n"/>
+      <c r="AO9" s="5" t="n"/>
+      <c r="AP9" s="5" t="n"/>
+      <c r="AQ9" s="5" t="inlineStr">
+        <is>
+          <t>Free 14-day Look Period</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Saholat Savings And Protection Plan</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="n"/>
+      <c r="J10" s="3" t="n"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="3" t="n"/>
+      <c r="N10" s="3" t="n"/>
+      <c r="O10" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Saholat Savings And Protection Plan</t>
+        </is>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Saholat Savings And Protection Plan</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="n"/>
+      <c r="R10" s="3" t="n"/>
+      <c r="S10" s="3" t="n"/>
+      <c r="T10" s="3" t="n"/>
+      <c r="U10" s="3" t="n"/>
+      <c r="V10" s="3" t="n"/>
+      <c r="W10" s="3" t="n"/>
+      <c r="X10" s="3" t="n"/>
+      <c r="Y10" s="3" t="n"/>
+      <c r="Z10" s="3" t="n"/>
+      <c r="AA10" s="3" t="n"/>
+      <c r="AB10" s="3" t="n"/>
+      <c r="AC10" s="3" t="n"/>
+      <c r="AD10" s="3" t="n"/>
+      <c r="AE10" s="3" t="n"/>
+      <c r="AF10" s="3" t="n"/>
+      <c r="AG10" s="3" t="n"/>
+      <c r="AH10" s="3" t="inlineStr">
+        <is>
+          <t>10-67 Y</t>
+        </is>
+      </c>
+      <c r="AI10" s="3" t="inlineStr">
+        <is>
+          <t>10-67 Years</t>
+        </is>
+      </c>
+      <c r="AJ10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="AK10" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="AL10" s="3" t="n"/>
+      <c r="AM10" s="3" t="n"/>
+      <c r="AN10" s="3" t="n"/>
+      <c r="AO10" s="3" t="n"/>
+      <c r="AP10" s="3" t="n"/>
+      <c r="AQ10" s="3" t="inlineStr">
+        <is>
+          <t>Free 14 Day Look Period</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Shifa Takaful Plan</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Yearly Renewable Hospitalization Plan</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Bankalfalah</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Bankalfalah</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Shifa Takaful Plan</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Shifa Takaful Plan</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="n"/>
+      <c r="R11" s="5" t="n"/>
+      <c r="S11" s="5" t="n"/>
+      <c r="T11" s="5" t="n"/>
+      <c r="U11" s="5" t="n"/>
+      <c r="V11" s="5" t="n"/>
+      <c r="W11" s="5" t="n"/>
+      <c r="X11" s="5" t="n"/>
+      <c r="Y11" s="5" t="n"/>
+      <c r="Z11" s="5" t="n"/>
+      <c r="AA11" s="5" t="n"/>
+      <c r="AB11" s="5" t="n"/>
+      <c r="AC11" s="5" t="n"/>
+      <c r="AD11" s="5" t="n">
+        <v>1.500003000005e+17</v>
+      </c>
+      <c r="AE11" s="5" t="n"/>
+      <c r="AF11" s="5" t="n"/>
+      <c r="AG11" s="5" t="n"/>
+      <c r="AH11" s="5" t="n"/>
+      <c r="AI11" s="5" t="n"/>
+      <c r="AJ11" s="5" t="n"/>
+      <c r="AK11" s="5" t="n"/>
+      <c r="AL11" s="5" t="n"/>
+      <c r="AM11" s="5" t="n"/>
+      <c r="AN11" s="5" t="n"/>
+      <c r="AO11" s="5" t="n"/>
+      <c r="AP11" s="5" t="n"/>
+      <c r="AQ11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Tadbeer Multipurpose Savings Plan</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Saving</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="n"/>
+      <c r="N12" s="3" t="n"/>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="n"/>
+      <c r="R12" s="3" t="n"/>
+      <c r="S12" s="3" t="n"/>
+      <c r="T12" s="3" t="n"/>
+      <c r="U12" s="3" t="n"/>
+      <c r="V12" s="3" t="n"/>
+      <c r="W12" s="3" t="n"/>
+      <c r="X12" s="3" t="n"/>
+      <c r="Y12" s="3" t="n"/>
+      <c r="Z12" s="3" t="n"/>
+      <c r="AA12" s="3" t="n"/>
+      <c r="AB12" s="3" t="n"/>
+      <c r="AC12" s="3" t="n"/>
+      <c r="AD12" s="3" t="n"/>
+      <c r="AE12" s="3" t="n"/>
+      <c r="AF12" s="3" t="n"/>
+      <c r="AG12" s="3" t="n"/>
+      <c r="AH12" s="3" t="inlineStr">
+        <is>
+          <t>10-65</t>
+        </is>
+      </c>
+      <c r="AI12" s="3" t="n"/>
+      <c r="AJ12" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="AK12" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="AL12" s="3" t="n"/>
+      <c r="AM12" s="3" t="n"/>
+      <c r="AN12" s="3" t="n"/>
+      <c r="AO12" s="3" t="n"/>
+      <c r="AP12" s="3" t="n"/>
+      <c r="AQ12" s="3" t="inlineStr">
+        <is>
+          <t>Free 14-day Look Period</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Uroos Marriage Plan</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Uroos Marriage Plan</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Uroos Marriage Plan</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
+      <c r="M13" s="5" t="n"/>
+      <c r="N13" s="5" t="n"/>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Uroos Marriage Plan</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Uroos Marriage Plan</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="5" t="n"/>
+      <c r="S13" s="5" t="n"/>
+      <c r="T13" s="5" t="n"/>
+      <c r="U13" s="5" t="n"/>
+      <c r="V13" s="5" t="n"/>
+      <c r="W13" s="5" t="n"/>
+      <c r="X13" s="5" t="n"/>
+      <c r="Y13" s="5" t="n"/>
+      <c r="Z13" s="5" t="n"/>
+      <c r="AA13" s="5" t="n"/>
+      <c r="AB13" s="5" t="n"/>
+      <c r="AC13" s="5" t="n"/>
+      <c r="AD13" s="5" t="n"/>
+      <c r="AE13" s="5" t="n"/>
+      <c r="AF13" s="5" t="n"/>
+      <c r="AG13" s="5" t="n"/>
+      <c r="AH13" s="5" t="n"/>
+      <c r="AI13" s="5" t="n"/>
+      <c r="AJ13" s="5" t="n"/>
+      <c r="AK13" s="5" t="n"/>
+      <c r="AL13" s="5" t="n"/>
+      <c r="AM13" s="5" t="n"/>
+      <c r="AN13" s="5" t="n"/>
+      <c r="AO13" s="5" t="n"/>
+      <c r="AP13" s="5" t="n"/>
+      <c r="AQ13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Zeenat Takaful Plan</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="3" t="n"/>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="3" t="n"/>
+      <c r="N14" s="3" t="n"/>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Zeenat Takaful Plan</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>IGI LIFE WTO Zeenat Takaful Plan</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="n"/>
+      <c r="R14" s="3" t="n"/>
+      <c r="S14" s="3" t="n"/>
+      <c r="T14" s="3" t="n"/>
+      <c r="U14" s="3" t="n"/>
+      <c r="V14" s="3" t="n"/>
+      <c r="W14" s="3" t="n"/>
+      <c r="X14" s="3" t="n"/>
+      <c r="Y14" s="3" t="n"/>
+      <c r="Z14" s="3" t="n"/>
+      <c r="AA14" s="3" t="n"/>
+      <c r="AB14" s="3" t="n"/>
+      <c r="AC14" s="3" t="n"/>
+      <c r="AD14" s="3" t="n"/>
+      <c r="AE14" s="3" t="n"/>
+      <c r="AF14" s="3" t="n"/>
+      <c r="AG14" s="3" t="n"/>
+      <c r="AH14" s="3" t="n"/>
+      <c r="AI14" s="3" t="n"/>
+      <c r="AJ14" s="3" t="n"/>
+      <c r="AK14" s="3" t="n"/>
+      <c r="AL14" s="3" t="n"/>
+      <c r="AM14" s="3" t="n"/>
+      <c r="AN14" s="3" t="n"/>
+      <c r="AO14" s="3" t="n"/>
+      <c r="AP14" s="3" t="n"/>
+      <c r="AQ14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>JUBILEE KAMIL TAKAFUL SAVINGS PLAN</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Savings</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="5" t="n"/>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>JUBILEE KAMIL TAKAFUL SAVINGS PLAN</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>JUBILEE KAMIL TAKAFUL SAVINGS PLAN</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="5" t="n"/>
+      <c r="S15" s="5" t="n"/>
+      <c r="T15" s="5" t="n"/>
+      <c r="U15" s="5" t="n"/>
+      <c r="V15" s="5" t="n"/>
+      <c r="W15" s="5" t="n"/>
+      <c r="X15" s="5" t="n"/>
+      <c r="Y15" s="5" t="n"/>
+      <c r="Z15" s="5" t="n"/>
+      <c r="AA15" s="5" t="n"/>
+      <c r="AB15" s="5" t="n"/>
+      <c r="AC15" s="5" t="n"/>
+      <c r="AD15" s="5" t="n"/>
+      <c r="AE15" s="5" t="n"/>
+      <c r="AF15" s="5" t="n"/>
+      <c r="AG15" s="5" t="n"/>
+      <c r="AH15" s="5" t="n"/>
+      <c r="AI15" s="5" t="n"/>
+      <c r="AJ15" s="5" t="n"/>
+      <c r="AK15" s="5" t="n"/>
+      <c r="AL15" s="5" t="n"/>
+      <c r="AM15" s="5" t="n"/>
+      <c r="AN15" s="5" t="n"/>
+      <c r="AO15" s="5" t="n"/>
+      <c r="AP15" s="5" t="n"/>
+      <c r="AQ15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>SLIC Tayyab Takaful Endowment Plan</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>IBG</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Banca Takaful</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Protection</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="n"/>
+      <c r="J16" s="3" t="n"/>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="3" t="n"/>
+      <c r="N16" s="3" t="n"/>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>SLIC Tayyab Takaful Endowment Plan</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>SLIC Tayyab Takaful Endowment Plan</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="n"/>
+      <c r="R16" s="3" t="n"/>
+      <c r="S16" s="3" t="n"/>
+      <c r="T16" s="3" t="n"/>
+      <c r="U16" s="3" t="n"/>
+      <c r="V16" s="3" t="n"/>
+      <c r="W16" s="3" t="n"/>
+      <c r="X16" s="3" t="n"/>
+      <c r="Y16" s="3" t="n"/>
+      <c r="Z16" s="3" t="n"/>
+      <c r="AA16" s="3" t="n"/>
+      <c r="AB16" s="3" t="n"/>
+      <c r="AC16" s="3" t="n"/>
+      <c r="AD16" s="3" t="n"/>
+      <c r="AE16" s="3" t="n"/>
+      <c r="AF16" s="3" t="n"/>
+      <c r="AG16" s="3" t="n"/>
+      <c r="AH16" s="3" t="n"/>
+      <c r="AI16" s="3" t="n"/>
+      <c r="AJ16" s="3" t="n"/>
+      <c r="AK16" s="3" t="n"/>
+      <c r="AL16" s="3" t="n"/>
+      <c r="AM16" s="3" t="n"/>
+      <c r="AN16" s="3" t="n"/>
+      <c r="AO16" s="3" t="n"/>
+      <c r="AP16" s="3" t="n"/>
+      <c r="AQ16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Home Loans</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>BNK</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>SBP Covid 19 Schemes</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 Annexure C</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 Annexure C</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
+      <c r="K17" s="5" t="n"/>
+      <c r="L17" s="5" t="n"/>
+      <c r="M17" s="5" t="n"/>
+      <c r="N17" s="5" t="n"/>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 Annexure C</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 Annexure C</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="5" t="n"/>
+      <c r="S17" s="5" t="n"/>
+      <c r="T17" s="5" t="n"/>
+      <c r="U17" s="5" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="V17" s="5" t="inlineStr">
+        <is>
+          <t>Cash</t>
+        </is>
+      </c>
+      <c r="W17" s="5" t="n"/>
+      <c r="X17" s="5" t="n"/>
+      <c r="Y17" s="5" t="n"/>
+      <c r="Z17" s="5" t="n"/>
+      <c r="AA17" s="5" t="n"/>
+      <c r="AB17" s="5" t="n"/>
+      <c r="AC17" s="5" t="inlineStr">
+        <is>
+          <t>0-50 Mn</t>
+        </is>
+      </c>
+      <c r="AD17" s="5" t="n"/>
+      <c r="AE17" s="5" t="n"/>
+      <c r="AF17" s="5" t="n"/>
+      <c r="AG17" s="5" t="n"/>
+      <c r="AH17" s="5" t="n"/>
+      <c r="AI17" s="5" t="n"/>
+      <c r="AJ17" s="5" t="n"/>
+      <c r="AK17" s="5" t="n"/>
+      <c r="AL17" s="5" t="n"/>
+      <c r="AM17" s="5" t="n"/>
+      <c r="AN17" s="5" t="n"/>
+      <c r="AO17" s="5" t="n"/>
+      <c r="AP17" s="5" t="n"/>
+      <c r="AQ17" s="5" t="inlineStr">
+        <is>
+          <t>Product Head- Secured Business Head-secured Segment Head Of Credit Operations Head Of Credit Risk Policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>SBP Financial Relief</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>BNK</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>SBP Covid 19 Schemes</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Deferral</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Consumer Finance Relief</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Salaried</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Salaried</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Salaried</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="n"/>
+      <c r="M18" s="3" t="n"/>
+      <c r="N18" s="3" t="n"/>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 SBP Financial Relief Consumers</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 SBP Financial Relief Consumers</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>Open To All</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>Financial Relief</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="n"/>
+      <c r="U18" s="3" t="n"/>
+      <c r="V18" s="3" t="n"/>
+      <c r="W18" s="3" t="n"/>
+      <c r="X18" s="3" t="n"/>
+      <c r="Y18" s="3" t="n"/>
+      <c r="Z18" s="3" t="n"/>
+      <c r="AA18" s="3" t="n"/>
+      <c r="AB18" s="3" t="n"/>
+      <c r="AC18" s="3" t="n"/>
+      <c r="AD18" s="3" t="n"/>
+      <c r="AE18" s="3" t="inlineStr">
+        <is>
+          <t>Consumer Products</t>
+        </is>
+      </c>
+      <c r="AF18" s="3" t="n"/>
+      <c r="AG18" s="3" t="n"/>
+      <c r="AH18" s="3" t="inlineStr">
+        <is>
+          <t>1 Y</t>
+        </is>
+      </c>
+      <c r="AI18" s="3" t="inlineStr">
+        <is>
+          <t>1 Year</t>
+        </is>
+      </c>
+      <c r="AJ18" s="3" t="n"/>
+      <c r="AK18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL18" s="3" t="n"/>
+      <c r="AM18" s="3" t="n"/>
+      <c r="AN18" s="3" t="n"/>
+      <c r="AO18" s="3" t="n"/>
+      <c r="AP18" s="3" t="n"/>
+      <c r="AQ18" s="3" t="inlineStr">
+        <is>
+          <t>Deferral Up To 1 Year; Rescheduling Up To 2 Years</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 Annexure B</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>BNK</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>SBP Covid 19 Schemes</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 Annexure B</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 Annexure B</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="5" t="n"/>
+      <c r="J19" s="5" t="n"/>
+      <c r="K19" s="5" t="n"/>
+      <c r="L19" s="5" t="n"/>
+      <c r="M19" s="5" t="n"/>
+      <c r="N19" s="5" t="n"/>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 Annexure B</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>SBP Schemes Covid-19 Annexure B</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="n"/>
+      <c r="R19" s="5" t="n"/>
+      <c r="S19" s="5" t="n"/>
+      <c r="T19" s="5" t="n"/>
+      <c r="U19" s="5" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+      <c r="V19" s="5" t="n"/>
+      <c r="W19" s="5" t="n"/>
+      <c r="X19" s="5" t="n"/>
+      <c r="Y19" s="5" t="n"/>
+      <c r="Z19" s="5" t="n"/>
+      <c r="AA19" s="5" t="n"/>
+      <c r="AB19" s="5" t="n"/>
+      <c r="AC19" s="5" t="n"/>
+      <c r="AD19" s="5" t="n"/>
+      <c r="AE19" s="5" t="inlineStr">
+        <is>
+          <t>SBS</t>
+        </is>
+      </c>
+      <c r="AF19" s="5" t="inlineStr">
+        <is>
+          <t>Markup</t>
+        </is>
+      </c>
+      <c r="AG19" s="5" t="inlineStr">
+        <is>
+          <t>APR</t>
+        </is>
+      </c>
+      <c r="AH19" s="5" t="inlineStr">
+        <is>
+          <t>3 Y</t>
+        </is>
+      </c>
+      <c r="AI19" s="5" t="inlineStr">
+        <is>
+          <t>3 Years</t>
+        </is>
+      </c>
+      <c r="AJ19" s="5" t="n"/>
+      <c r="AK19" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL19" s="5" t="n"/>
+      <c r="AM19" s="5" t="n"/>
+      <c r="AN19" s="5" t="n"/>
+      <c r="AO19" s="5" t="n"/>
+      <c r="AP19" s="5" t="n"/>
+      <c r="AQ19" s="5" t="inlineStr">
+        <is>
+          <t>0% Markup, Extend Tenure Up To 3 Years</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AQ1"/>

</xml_diff>